<commit_message>
Actualizar a la version final del laboratorio
Agrega presentacion, ENTREGABLES, estrategia en .docx, matriz actualizada y capturas de evidencias. Servicios, gateway y coleccion sin cambios.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/matriz-casos-de-prueba.xlsx
+++ b/docs/matriz-casos-de-prueba.xlsx
@@ -20,12 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="114">
   <si>
     <t xml:space="preserve">Matriz de casos de prueba — Grupo 4 · Arquitectura con API Gateway (Kong)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leyenda: las celdas amarillas (Resultado obtenido y Estado) se diligencian después de ejecutar las pruebas. Estado: Aprobado / Fallido.</t>
   </si>
   <si>
     <t xml:space="preserve">Identificador</t>
@@ -96,7 +93,13 @@
     <t xml:space="preserve">200 OK; arreglo de productos con id, nombre, precio, stock; cabecera X-Request-ID.</t>
   </si>
   <si>
+    <t xml:space="preserve">200 OK en 264 ms. Arreglo con 3 productos (id, nombre, precio, stock). Cabecera X-Request-ID presente. Test Results: 3/3 PASSED.</t>
+  </si>
+  <si>
     <t xml:space="preserve">reporte-funcional.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprobado</t>
   </si>
   <si>
     <t xml:space="preserve">César</t>
@@ -125,6 +128,9 @@
   </si>
   <si>
     <t xml:space="preserve">200 OK; arreglo de pedidos; cabecera X-Kong-Upstream-Latency presente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK en 169 ms. Arreglo vacío [] (aún no hay pedidos creados). Cabecera X-Kong-Upstream-Latency presente. Test Results: 3/3 PASSED.</t>
   </si>
   <si>
     <t xml:space="preserve">CP-03</t>
@@ -153,6 +159,9 @@
     <t xml:space="preserve">401 Unauthorized; mensaje 'No API key found in request' de Kong; sin cabecera X-Kong-Upstream-Latency.</t>
   </si>
   <si>
+    <t xml:space="preserve">401 Unauthorized en 20 ms. Mensaje de Kong "No API key found in request". Sin cabecera X-Kong-Upstream-Latency (la solicitud no llegó al servicio). Test Results: 2/2 PASSED.</t>
+  </si>
+  <si>
     <t xml:space="preserve">reporte-funcional.html + log-servicios.txt</t>
   </si>
   <si>
@@ -181,6 +190,9 @@
     <t xml:space="preserve">404 Not Found; mensaje 'no Route matched with those values'.</t>
   </si>
   <si>
+    <t xml:space="preserve">404 Not Found en 165 ms. Mensaje de Kong "no Route matched with those values". Test Results: 2/2 PASSED.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CP-05</t>
   </si>
   <si>
@@ -201,6 +213,9 @@
   </si>
   <si>
     <t xml:space="preserve">400 Bad Request; error DATOS_INVALIDOS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">400 Bad Request en 272 ms. error DATOS_INVALIDOS con detalle "productoId y cantidad deben ser enteros y cantidad &gt; 0". El error del servicio Pedidos se propagó por Kong. Test Results: 2/2 PASSED.</t>
   </si>
   <si>
     <t xml:space="preserve">Paulina</t>
@@ -232,6 +247,9 @@
     <t xml:space="preserve">422 Unprocessable Entity; error PRODUCTO_NO_EXISTE.</t>
   </si>
   <si>
+    <t xml:space="preserve">422 Unprocessable Entity en 228 ms. error PRODUCTO_NO_EXISTE, productoId 99. Pedidos consultó a Productos, que respondió 404, y Pedidos lo tradujo a 422. Test Results: 2/2 PASSED</t>
+  </si>
+  <si>
     <t xml:space="preserve">CP-07</t>
   </si>
   <si>
@@ -258,6 +276,9 @@
   <si>
     <t xml:space="preserve">1) 201 Created, total = 360000, estado CREADO.
 2) 200 OK con el mismo id y estado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) 201 Created en 169 ms: pedido id 1, total 360000, estado CREADO. 2) 200 OK en 23 ms: mismo id, productoId, cantidad, total y estado. Test Results: 2/2 PASSED en ambos pasos.</t>
   </si>
   <si>
     <t xml:space="preserve">CP-08</t>
@@ -291,7 +312,11 @@
 /api/productos: 200 (aislamiento).</t>
   </si>
   <si>
-    <t xml:space="preserve">reporte-servicio-caido.html + log-gateway.txt</t>
+    <t xml:space="preserve">Con Pedidos detenido: GET /api/pedidos → 504 Gateway Timeout en 2,09 s (Kong: "upstream timed out while connecting", corta el connect_timeout de 2 s). GET /api/productos → 200 OK en 132 ms (aislamiento correcto). Pedidos se recuperó al encenderlo.
+HALLAZGO H-01: en la primera ejecución la respuesta fue 503 "name resolution failed" en 12,08 s, fuera del criterio de 5 s (esa corrida no cumplió). Causa probable: al detener el contenedor, el DNS interno de Docker deja de resolver "pedidos" y Kong espera al resolvedor DNS. En la repetición Kong ya tenía la IP en caché y falló al conectar en 2 s. Mejora propuesta: ajustar los tiempos del resolvedor DNS de Kong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reporte-servicio-caido.html + log-gateway.txt (líneas [error] upstream timed out)</t>
   </si>
   <si>
     <t xml:space="preserve">Camilo</t>
@@ -319,6 +344,9 @@
     <t xml:space="preserve">504 Gateway Timeout en menos de 4,5 s.</t>
   </si>
   <si>
+    <t xml:space="preserve">504 Gateway Timeout en 3,03 s. Mensaje de Kong "The upstream server is timing out". El gateway cortó a los 3 s (read_timeout) sin esperar los 5 s del servicio. Test Results: 2/2 PASSED.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CP-10</t>
   </si>
   <si>
@@ -339,6 +367,9 @@
   </si>
   <si>
     <t xml:space="preserve">Primeras ~5 en 200; las siguientes en 429 Too Many Requests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 solicitudes seguidas a GET /api/productos con el script (2 oct 2026, 10:39:51): 5 respondieron 200 y 5 respondieron 429 (Too Many Requests). Secuencia: 200,200,200,200,200,429,429,429,429,429. Cabeceras RateLimit-Limit: 5 y RateLimit-Remaining confirman el contador. Observación: con un bucle manual de curl.exe salió 200×5, 429×3, 200×2, porque el bucle tardó más de 1 s y las últimas solicitudes cayeron en una ventana nueva; no es un defecto.</t>
   </si>
   <si>
     <t xml:space="preserve">resultado-rate-limit.txt</t>
@@ -357,10 +388,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -402,9 +432,8 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -427,24 +456,12 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -496,7 +513,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -509,15 +526,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -526,10 +539,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -562,7 +571,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -592,7 +601,7 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1F3864"/>
+      <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
@@ -786,9 +795,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
@@ -800,464 +809,496 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="3" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="5"/>
       <c r="K5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="5"/>
+      <c r="L5" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M5" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="5"/>
+        <v>34</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="K6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="5"/>
+      <c r="L6" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M6" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" s="5"/>
       <c r="M7" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J8" s="5"/>
+        <v>53</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="K8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="5"/>
+      <c r="L8" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M8" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="J9" s="5"/>
+        <v>61</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>62</v>
+      </c>
       <c r="K9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L9" s="5"/>
+      <c r="L9" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M9" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="G10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="L10" s="5"/>
-      <c r="M10" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J11" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="K11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="5"/>
+      <c r="L11" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M11" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J12" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="K12" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="L12" s="5"/>
-      <c r="M12" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="D13" s="4" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" s="5"/>
+        <v>100</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>101</v>
+      </c>
       <c r="K13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L13" s="5"/>
+      <c r="L13" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M13" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="J14" s="5"/>
+        <v>108</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="K14" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="L14" s="5"/>
+        <v>110</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="M14" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B16" s="7" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="6" t="n">
         <f aca="false">COUNTIF(L5:L14,"Aprobado")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B17" s="7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="6" t="n">
         <f aca="false">COUNTIF(L5:L14,"Fallido")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" s="8" t="n">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="6" t="n">
         <f aca="false">IFERROR(B16/(B16+B17),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L14" type="list">
-      <formula1>"Aprobado,Fallido"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>